<commit_message>
Realign resource publication to OneDrive Resource authority.
OneDrive Resource is now the authoritative source for all six resource workbooks; staging and public paths are distribution copies only. GHG FY2568 moves to 1.6GreenHouseGas2025.xlsx (231.23 tCO2e), with publication manifest, validation gates, and audit matrices. FY2569 form bulk publish deferred to follow-up PR.
</commit_message>
<xml_diff>
--- a/data/staging/source/1.4paper.xlsx
+++ b/data/staging/source/1.4paper.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maejo365-my.sharepoint.com/personal/researchmju_mju_ac_th/Documents/RAE-Document-Center/07-GreenOffice/Resource/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="8_{2CA96BB9-9D5B-4BBD-A3B8-9B00E6CB572B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B247F63-5867-4A69-84D3-954725F62B44}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="8_{2CA96BB9-9D5B-4BBD-A3B8-9B00E6CB572B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDB2E810-31E1-46B5-8063-9EA17E6AA1AB}"/>
   <bookViews>
     <workbookView xWindow="23880" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="3" xr2:uid="{598E5E77-AA4E-4BC9-9064-64F7A2894463}"/>
   </bookViews>
@@ -1602,33 +1602,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="27" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="13" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="23" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="28" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="27" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="13" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="23" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="28" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="19" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="8" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
@@ -1637,9 +1610,6 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="8" borderId="13" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="19" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -1659,11 +1629,38 @@
     <xf numFmtId="0" fontId="20" fillId="7" borderId="13" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="19" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="13" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="27" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="23" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="28" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="27" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="13" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="23" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="28" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="19" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1680,20 +1677,23 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2017,7 +2017,7 @@
                   <c:v>224.10000000000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>30.402000000000001</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -2032,7 +2032,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>103.31325</c:v>
+                  <c:v>105.84675</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7438,7 +7438,7 @@
                   <c:v>2.3840425531914895</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.32342553191489365</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -7453,7 +7453,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0990771276595743</c:v>
+                  <c:v>1.1260292553191489</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8330,7 +8330,7 @@
                   <c:v>2197.7999999999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1239.759</c:v>
+                  <c:v>1270.1610000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8683,7 +8683,7 @@
                   <c:v>23.134736842105266</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.188925531914895</c:v>
+                  <c:v>13.512351063829788</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -19344,44 +19344,44 @@
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" ht="23.1" customHeight="1">
-      <c r="A2" s="140" t="s">
+      <c r="A2" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="140"/>
-      <c r="C2" s="140"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="140"/>
-      <c r="F2" s="140"/>
-      <c r="G2" s="140"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="140"/>
-      <c r="J2" s="140"/>
-      <c r="K2" s="140"/>
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="139"/>
+      <c r="I2" s="139"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="139"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12" s="6" customFormat="1" ht="21.6" customHeight="1">
-      <c r="A3" s="141" t="s">
+      <c r="A3" s="140" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="142" t="s">
+      <c r="B3" s="141" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="142"/>
-      <c r="E3" s="142"/>
-      <c r="F3" s="142" t="s">
+      <c r="C3" s="141"/>
+      <c r="D3" s="141"/>
+      <c r="E3" s="141"/>
+      <c r="F3" s="141" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="142"/>
-      <c r="H3" s="142"/>
-      <c r="I3" s="142"/>
-      <c r="J3" s="142" t="s">
+      <c r="G3" s="141"/>
+      <c r="H3" s="141"/>
+      <c r="I3" s="141"/>
+      <c r="J3" s="141" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="142"/>
+      <c r="K3" s="141"/>
     </row>
     <row r="4" spans="1:12" s="6" customFormat="1" ht="45.95" customHeight="1">
-      <c r="A4" s="141"/>
+      <c r="A4" s="140"/>
       <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
@@ -19746,23 +19746,23 @@
       </c>
       <c r="G12" s="10">
         <f>แต่ละหน่วยงาน!J128</f>
-        <v>0</v>
+        <v>30.402000000000001</v>
       </c>
       <c r="H12" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1276.884</v>
       </c>
       <c r="I12" s="9">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.32342553191489365</v>
       </c>
       <c r="J12" s="11">
         <f t="shared" si="3"/>
-        <v>-1</v>
+        <v>-0.85281045751633999</v>
       </c>
       <c r="K12" s="12">
         <f t="shared" si="4"/>
-        <v>-1</v>
+        <v>-0.85124461131970508</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="24.95" customHeight="1">
@@ -19967,23 +19967,23 @@
       </c>
       <c r="G17" s="9">
         <f t="shared" si="6"/>
-        <v>103.31325</v>
+        <v>105.84675</v>
       </c>
       <c r="H17" s="9">
         <f t="shared" si="6"/>
-        <v>4339.1565000000001</v>
+        <v>4445.5634999999993</v>
       </c>
       <c r="I17" s="9">
         <f>G17/F17</f>
-        <v>1.0990771276595743</v>
+        <v>1.1260292553191489</v>
       </c>
       <c r="J17" s="11">
         <f>(G17-C17)/C17</f>
-        <v>-0.43590909090909086</v>
+        <v>-0.42207616707616702</v>
       </c>
       <c r="K17" s="12">
         <f>(I17-E17)/E17</f>
-        <v>-0.42990812379110266</v>
+        <v>-0.41592804119399873</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="24.95" customHeight="1">
@@ -20012,23 +20012,23 @@
       </c>
       <c r="G18" s="9">
         <f t="shared" si="7"/>
-        <v>1239.759</v>
+        <v>1270.1610000000001</v>
       </c>
       <c r="H18" s="9">
         <f t="shared" si="7"/>
-        <v>52069.877999999997</v>
+        <v>53346.761999999995</v>
       </c>
       <c r="I18" s="9">
         <f t="shared" si="7"/>
-        <v>13.188925531914895</v>
+        <v>13.512351063829788</v>
       </c>
       <c r="J18" s="11">
         <f t="shared" si="3"/>
-        <v>-0.43590909090909086</v>
+        <v>-0.42207616707616696</v>
       </c>
       <c r="K18" s="12">
         <f t="shared" si="4"/>
-        <v>-0.42990812379110249</v>
+        <v>-0.41592804119399868</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="11.45" customHeight="1">
@@ -20072,76 +20072,76 @@
     </row>
     <row r="40" spans="1:12" ht="21.95" customHeight="1"/>
     <row r="43" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A43" s="143" t="s">
+      <c r="A43" s="142" t="s">
         <v>28</v>
       </c>
-      <c r="B43" s="143"/>
-      <c r="C43" s="143"/>
-      <c r="D43" s="143"/>
-      <c r="E43" s="143"/>
-      <c r="F43" s="143"/>
-      <c r="G43" s="143"/>
-      <c r="H43" s="143"/>
-      <c r="I43" s="143"/>
-      <c r="J43" s="143"/>
-      <c r="K43" s="143"/>
-      <c r="L43" s="143"/>
+      <c r="B43" s="142"/>
+      <c r="C43" s="142"/>
+      <c r="D43" s="142"/>
+      <c r="E43" s="142"/>
+      <c r="F43" s="142"/>
+      <c r="G43" s="142"/>
+      <c r="H43" s="142"/>
+      <c r="I43" s="142"/>
+      <c r="J43" s="142"/>
+      <c r="K43" s="142"/>
+      <c r="L43" s="142"/>
     </row>
     <row r="44" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A44" s="143"/>
-      <c r="B44" s="143"/>
-      <c r="C44" s="143"/>
-      <c r="D44" s="143"/>
-      <c r="E44" s="143"/>
-      <c r="F44" s="143"/>
-      <c r="G44" s="143"/>
-      <c r="H44" s="143"/>
-      <c r="I44" s="143"/>
-      <c r="J44" s="143"/>
-      <c r="K44" s="143"/>
-      <c r="L44" s="143"/>
+      <c r="A44" s="142"/>
+      <c r="B44" s="142"/>
+      <c r="C44" s="142"/>
+      <c r="D44" s="142"/>
+      <c r="E44" s="142"/>
+      <c r="F44" s="142"/>
+      <c r="G44" s="142"/>
+      <c r="H44" s="142"/>
+      <c r="I44" s="142"/>
+      <c r="J44" s="142"/>
+      <c r="K44" s="142"/>
+      <c r="L44" s="142"/>
     </row>
     <row r="45" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A45" s="143"/>
-      <c r="B45" s="143"/>
-      <c r="C45" s="143"/>
-      <c r="D45" s="143"/>
-      <c r="E45" s="143"/>
-      <c r="F45" s="143"/>
-      <c r="G45" s="143"/>
-      <c r="H45" s="143"/>
-      <c r="I45" s="143"/>
-      <c r="J45" s="143"/>
-      <c r="K45" s="143"/>
-      <c r="L45" s="143"/>
+      <c r="A45" s="142"/>
+      <c r="B45" s="142"/>
+      <c r="C45" s="142"/>
+      <c r="D45" s="142"/>
+      <c r="E45" s="142"/>
+      <c r="F45" s="142"/>
+      <c r="G45" s="142"/>
+      <c r="H45" s="142"/>
+      <c r="I45" s="142"/>
+      <c r="J45" s="142"/>
+      <c r="K45" s="142"/>
+      <c r="L45" s="142"/>
     </row>
     <row r="46" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A46" s="143"/>
-      <c r="B46" s="143"/>
-      <c r="C46" s="143"/>
-      <c r="D46" s="143"/>
-      <c r="E46" s="143"/>
-      <c r="F46" s="143"/>
-      <c r="G46" s="143"/>
-      <c r="H46" s="143"/>
-      <c r="I46" s="143"/>
-      <c r="J46" s="143"/>
-      <c r="K46" s="143"/>
-      <c r="L46" s="143"/>
+      <c r="A46" s="142"/>
+      <c r="B46" s="142"/>
+      <c r="C46" s="142"/>
+      <c r="D46" s="142"/>
+      <c r="E46" s="142"/>
+      <c r="F46" s="142"/>
+      <c r="G46" s="142"/>
+      <c r="H46" s="142"/>
+      <c r="I46" s="142"/>
+      <c r="J46" s="142"/>
+      <c r="K46" s="142"/>
+      <c r="L46" s="142"/>
     </row>
     <row r="47" spans="1:12" ht="39.950000000000003" customHeight="1">
-      <c r="A47" s="143"/>
-      <c r="B47" s="143"/>
-      <c r="C47" s="143"/>
-      <c r="D47" s="143"/>
-      <c r="E47" s="143"/>
-      <c r="F47" s="143"/>
-      <c r="G47" s="143"/>
-      <c r="H47" s="143"/>
-      <c r="I47" s="143"/>
-      <c r="J47" s="143"/>
-      <c r="K47" s="143"/>
-      <c r="L47" s="143"/>
+      <c r="A47" s="142"/>
+      <c r="B47" s="142"/>
+      <c r="C47" s="142"/>
+      <c r="D47" s="142"/>
+      <c r="E47" s="142"/>
+      <c r="F47" s="142"/>
+      <c r="G47" s="142"/>
+      <c r="H47" s="142"/>
+      <c r="I47" s="142"/>
+      <c r="J47" s="142"/>
+      <c r="K47" s="142"/>
+      <c r="L47" s="142"/>
     </row>
     <row r="48" spans="1:12" ht="38.450000000000003" customHeight="1">
       <c r="A48" s="17"/>
@@ -20162,20 +20162,20 @@
       <c r="L48" s="17"/>
     </row>
     <row r="49" spans="1:12" ht="42" customHeight="1">
-      <c r="A49" s="144" t="s">
+      <c r="A49" s="143" t="s">
         <v>31</v>
       </c>
-      <c r="B49" s="144"/>
-      <c r="C49" s="144"/>
-      <c r="D49" s="144"/>
-      <c r="E49" s="144"/>
-      <c r="F49" s="144"/>
-      <c r="G49" s="144"/>
-      <c r="H49" s="144"/>
-      <c r="I49" s="144"/>
-      <c r="J49" s="144"/>
-      <c r="K49" s="144"/>
-      <c r="L49" s="144"/>
+      <c r="B49" s="143"/>
+      <c r="C49" s="143"/>
+      <c r="D49" s="143"/>
+      <c r="E49" s="143"/>
+      <c r="F49" s="143"/>
+      <c r="G49" s="143"/>
+      <c r="H49" s="143"/>
+      <c r="I49" s="143"/>
+      <c r="J49" s="143"/>
+      <c r="K49" s="143"/>
+      <c r="L49" s="143"/>
     </row>
     <row r="50" spans="1:12" s="21" customFormat="1" ht="30" customHeight="1">
       <c r="A50" s="20" t="s">
@@ -20214,10 +20214,10 @@
       <c r="L51" s="24"/>
     </row>
     <row r="52" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A52" s="139" t="s">
+      <c r="A52" s="144" t="s">
         <v>34</v>
       </c>
-      <c r="B52" s="139"/>
+      <c r="B52" s="144"/>
       <c r="C52" s="25"/>
       <c r="D52" s="26"/>
       <c r="E52" s="24"/>
@@ -20282,10 +20282,10 @@
       <c r="L55" s="24"/>
     </row>
     <row r="56" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A56" s="139" t="s">
+      <c r="A56" s="144" t="s">
         <v>34</v>
       </c>
-      <c r="B56" s="139"/>
+      <c r="B56" s="144"/>
       <c r="C56" s="25"/>
       <c r="D56" s="26"/>
       <c r="E56" s="24"/>
@@ -20622,10 +20622,10 @@
       <c r="L75" s="24"/>
     </row>
     <row r="76" spans="1:12" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A76" s="139" t="s">
+      <c r="A76" s="144" t="s">
         <v>34</v>
       </c>
-      <c r="B76" s="139"/>
+      <c r="B76" s="144"/>
       <c r="C76" s="25"/>
       <c r="D76" s="26"/>
       <c r="E76" s="24"/>
@@ -20690,10 +20690,10 @@
       <c r="L79" s="24"/>
     </row>
     <row r="80" spans="1:12" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A80" s="139" t="s">
+      <c r="A80" s="144" t="s">
         <v>34</v>
       </c>
-      <c r="B80" s="139"/>
+      <c r="B80" s="144"/>
       <c r="C80" s="25"/>
       <c r="D80" s="26"/>
       <c r="E80" s="24"/>
@@ -21025,6 +21025,13 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A96:B96"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="A80:B80"/>
+    <mergeCell ref="A84:B84"/>
+    <mergeCell ref="A88:B88"/>
+    <mergeCell ref="A92:B92"/>
     <mergeCell ref="A68:B68"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A3:A4"/>
@@ -21037,13 +21044,6 @@
     <mergeCell ref="A56:B56"/>
     <mergeCell ref="A60:B60"/>
     <mergeCell ref="A64:B64"/>
-    <mergeCell ref="A96:B96"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="A80:B80"/>
-    <mergeCell ref="A84:B84"/>
-    <mergeCell ref="A88:B88"/>
-    <mergeCell ref="A92:B92"/>
   </mergeCells>
   <pageMargins left="0.2" right="0.18" top="0.3" bottom="0.23" header="0.24" footer="0.23"/>
   <pageSetup paperSize="9" scale="68" orientation="portrait" horizontalDpi="4294967293" verticalDpi="1200" r:id="rId1"/>
@@ -21093,44 +21093,44 @@
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" ht="21" customHeight="1">
-      <c r="A2" s="140" t="s">
+      <c r="A2" s="139" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="140"/>
-      <c r="C2" s="140"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="140"/>
-      <c r="F2" s="140"/>
-      <c r="G2" s="140"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="140"/>
-      <c r="J2" s="140"/>
-      <c r="K2" s="140"/>
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="139"/>
+      <c r="I2" s="139"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="139"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12" s="6" customFormat="1" ht="21.6" customHeight="1">
-      <c r="A3" s="141" t="s">
+      <c r="A3" s="140" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="142" t="s">
+      <c r="B3" s="141" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="142"/>
-      <c r="E3" s="142"/>
-      <c r="F3" s="142" t="s">
+      <c r="C3" s="141"/>
+      <c r="D3" s="141"/>
+      <c r="E3" s="141"/>
+      <c r="F3" s="141" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="142"/>
-      <c r="H3" s="142"/>
-      <c r="I3" s="142"/>
-      <c r="J3" s="142" t="s">
+      <c r="G3" s="141"/>
+      <c r="H3" s="141"/>
+      <c r="I3" s="141"/>
+      <c r="J3" s="141" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="142"/>
+      <c r="K3" s="141"/>
     </row>
     <row r="4" spans="1:12" s="6" customFormat="1" ht="54" customHeight="1">
-      <c r="A4" s="141"/>
+      <c r="A4" s="140"/>
       <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
@@ -21765,99 +21765,99 @@
     </row>
     <row r="40" spans="1:17" ht="21.95" customHeight="1"/>
     <row r="43" spans="1:17" ht="21.75" customHeight="1">
-      <c r="A43" s="148" t="s">
+      <c r="A43" s="146" t="s">
         <v>56</v>
       </c>
-      <c r="B43" s="143"/>
-      <c r="C43" s="143"/>
-      <c r="D43" s="143"/>
-      <c r="E43" s="143"/>
-      <c r="F43" s="143"/>
-      <c r="G43" s="143"/>
-      <c r="H43" s="143"/>
-      <c r="I43" s="143"/>
-      <c r="J43" s="143"/>
-      <c r="K43" s="143"/>
-      <c r="L43" s="143"/>
+      <c r="B43" s="142"/>
+      <c r="C43" s="142"/>
+      <c r="D43" s="142"/>
+      <c r="E43" s="142"/>
+      <c r="F43" s="142"/>
+      <c r="G43" s="142"/>
+      <c r="H43" s="142"/>
+      <c r="I43" s="142"/>
+      <c r="J43" s="142"/>
+      <c r="K43" s="142"/>
+      <c r="L43" s="142"/>
     </row>
     <row r="44" spans="1:17" ht="21.75" customHeight="1">
-      <c r="A44" s="143"/>
-      <c r="B44" s="143"/>
-      <c r="C44" s="143"/>
-      <c r="D44" s="143"/>
-      <c r="E44" s="143"/>
-      <c r="F44" s="143"/>
-      <c r="G44" s="143"/>
-      <c r="H44" s="143"/>
-      <c r="I44" s="143"/>
-      <c r="J44" s="143"/>
-      <c r="K44" s="143"/>
-      <c r="L44" s="143"/>
+      <c r="A44" s="142"/>
+      <c r="B44" s="142"/>
+      <c r="C44" s="142"/>
+      <c r="D44" s="142"/>
+      <c r="E44" s="142"/>
+      <c r="F44" s="142"/>
+      <c r="G44" s="142"/>
+      <c r="H44" s="142"/>
+      <c r="I44" s="142"/>
+      <c r="J44" s="142"/>
+      <c r="K44" s="142"/>
+      <c r="L44" s="142"/>
       <c r="N44" s="33"/>
       <c r="O44" s="33"/>
       <c r="P44" s="33"/>
       <c r="Q44" s="33"/>
     </row>
     <row r="45" spans="1:17" ht="21.75" customHeight="1">
-      <c r="A45" s="143"/>
-      <c r="B45" s="143"/>
-      <c r="C45" s="143"/>
-      <c r="D45" s="143"/>
-      <c r="E45" s="143"/>
-      <c r="F45" s="143"/>
-      <c r="G45" s="143"/>
-      <c r="H45" s="143"/>
-      <c r="I45" s="143"/>
-      <c r="J45" s="143"/>
-      <c r="K45" s="143"/>
-      <c r="L45" s="143"/>
+      <c r="A45" s="142"/>
+      <c r="B45" s="142"/>
+      <c r="C45" s="142"/>
+      <c r="D45" s="142"/>
+      <c r="E45" s="142"/>
+      <c r="F45" s="142"/>
+      <c r="G45" s="142"/>
+      <c r="H45" s="142"/>
+      <c r="I45" s="142"/>
+      <c r="J45" s="142"/>
+      <c r="K45" s="142"/>
+      <c r="L45" s="142"/>
       <c r="P45" s="33"/>
       <c r="Q45" s="33"/>
     </row>
     <row r="46" spans="1:17" ht="21.75" customHeight="1">
-      <c r="A46" s="143"/>
-      <c r="B46" s="143"/>
-      <c r="C46" s="143"/>
-      <c r="D46" s="143"/>
-      <c r="E46" s="143"/>
-      <c r="F46" s="143"/>
-      <c r="G46" s="143"/>
-      <c r="H46" s="143"/>
-      <c r="I46" s="143"/>
-      <c r="J46" s="143"/>
-      <c r="K46" s="143"/>
-      <c r="L46" s="143"/>
+      <c r="A46" s="142"/>
+      <c r="B46" s="142"/>
+      <c r="C46" s="142"/>
+      <c r="D46" s="142"/>
+      <c r="E46" s="142"/>
+      <c r="F46" s="142"/>
+      <c r="G46" s="142"/>
+      <c r="H46" s="142"/>
+      <c r="I46" s="142"/>
+      <c r="J46" s="142"/>
+      <c r="K46" s="142"/>
+      <c r="L46" s="142"/>
       <c r="P46" s="33"/>
     </row>
     <row r="47" spans="1:17" ht="78.75" customHeight="1">
-      <c r="A47" s="143"/>
-      <c r="B47" s="143"/>
-      <c r="C47" s="143"/>
-      <c r="D47" s="143"/>
-      <c r="E47" s="143"/>
-      <c r="F47" s="143"/>
-      <c r="G47" s="143"/>
-      <c r="H47" s="143"/>
-      <c r="I47" s="143"/>
-      <c r="J47" s="143"/>
-      <c r="K47" s="143"/>
-      <c r="L47" s="143"/>
+      <c r="A47" s="142"/>
+      <c r="B47" s="142"/>
+      <c r="C47" s="142"/>
+      <c r="D47" s="142"/>
+      <c r="E47" s="142"/>
+      <c r="F47" s="142"/>
+      <c r="G47" s="142"/>
+      <c r="H47" s="142"/>
+      <c r="I47" s="142"/>
+      <c r="J47" s="142"/>
+      <c r="K47" s="142"/>
+      <c r="L47" s="142"/>
     </row>
     <row r="48" spans="1:17" ht="42" customHeight="1">
-      <c r="A48" s="149" t="s">
+      <c r="A48" s="147" t="s">
         <v>57</v>
       </c>
-      <c r="B48" s="149"/>
-      <c r="C48" s="149"/>
-      <c r="D48" s="149"/>
-      <c r="E48" s="149"/>
-      <c r="F48" s="149"/>
-      <c r="G48" s="149"/>
-      <c r="H48" s="149"/>
-      <c r="I48" s="149"/>
-      <c r="J48" s="149"/>
-      <c r="K48" s="149"/>
-      <c r="L48" s="149"/>
+      <c r="B48" s="147"/>
+      <c r="C48" s="147"/>
+      <c r="D48" s="147"/>
+      <c r="E48" s="147"/>
+      <c r="F48" s="147"/>
+      <c r="G48" s="147"/>
+      <c r="H48" s="147"/>
+      <c r="I48" s="147"/>
+      <c r="J48" s="147"/>
+      <c r="K48" s="147"/>
+      <c r="L48" s="147"/>
     </row>
     <row r="49" spans="1:12" s="21" customFormat="1" ht="30" customHeight="1">
       <c r="A49" s="145" t="s">
@@ -21883,10 +21883,10 @@
       <c r="C50" s="35"/>
     </row>
     <row r="51" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A51" s="147" t="s">
+      <c r="A51" s="148" t="s">
         <v>60</v>
       </c>
-      <c r="B51" s="147"/>
+      <c r="B51" s="148"/>
       <c r="C51" s="34" t="s">
         <v>61</v>
       </c>
@@ -21924,10 +21924,10 @@
       <c r="D54" s="34"/>
     </row>
     <row r="55" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A55" s="147" t="s">
+      <c r="A55" s="148" t="s">
         <v>34</v>
       </c>
-      <c r="B55" s="147"/>
+      <c r="B55" s="148"/>
       <c r="C55" s="34" t="s">
         <v>61</v>
       </c>
@@ -21965,10 +21965,10 @@
       <c r="D58" s="34"/>
     </row>
     <row r="59" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A59" s="146" t="s">
+      <c r="A59" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="146"/>
+      <c r="B59" s="149"/>
       <c r="C59" s="34" t="s">
         <v>66</v>
       </c>
@@ -22008,10 +22008,10 @@
       <c r="D62" s="34"/>
     </row>
     <row r="63" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A63" s="146" t="s">
+      <c r="A63" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B63" s="146"/>
+      <c r="B63" s="149"/>
       <c r="C63" s="34" t="s">
         <v>66</v>
       </c>
@@ -22051,10 +22051,10 @@
       <c r="D66" s="34"/>
     </row>
     <row r="67" spans="1:13" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A67" s="146" t="s">
+      <c r="A67" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B67" s="146"/>
+      <c r="B67" s="149"/>
       <c r="C67" s="34" t="s">
         <v>61</v>
       </c>
@@ -22091,10 +22091,10 @@
       <c r="D70" s="34"/>
     </row>
     <row r="71" spans="1:13" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A71" s="146" t="s">
+      <c r="A71" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B71" s="146"/>
+      <c r="B71" s="149"/>
       <c r="C71" s="34" t="s">
         <v>66</v>
       </c>
@@ -22135,21 +22135,21 @@
       <c r="C74" s="35"/>
     </row>
     <row r="75" spans="1:13" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A75" s="147" t="s">
+      <c r="A75" s="148" t="s">
         <v>34</v>
       </c>
-      <c r="B75" s="147"/>
-      <c r="C75" s="146" t="s">
+      <c r="B75" s="148"/>
+      <c r="C75" s="149" t="s">
         <v>66</v>
       </c>
-      <c r="D75" s="146"/>
-      <c r="E75" s="146"/>
-      <c r="F75" s="146"/>
-      <c r="G75" s="146"/>
-      <c r="H75" s="146"/>
-      <c r="I75" s="146"/>
-      <c r="J75" s="146"/>
-      <c r="K75" s="146"/>
+      <c r="D75" s="149"/>
+      <c r="E75" s="149"/>
+      <c r="F75" s="149"/>
+      <c r="G75" s="149"/>
+      <c r="H75" s="149"/>
+      <c r="I75" s="149"/>
+      <c r="J75" s="149"/>
+      <c r="K75" s="149"/>
     </row>
     <row r="76" spans="1:13" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A76" s="34" t="s">
@@ -22185,23 +22185,23 @@
       <c r="D78" s="34"/>
     </row>
     <row r="79" spans="1:13" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A79" s="147" t="s">
+      <c r="A79" s="148" t="s">
         <v>34</v>
       </c>
-      <c r="B79" s="147"/>
-      <c r="C79" s="146" t="s">
+      <c r="B79" s="148"/>
+      <c r="C79" s="149" t="s">
         <v>66</v>
       </c>
-      <c r="D79" s="146"/>
-      <c r="E79" s="146"/>
-      <c r="F79" s="146"/>
-      <c r="G79" s="146"/>
-      <c r="H79" s="146"/>
-      <c r="I79" s="146"/>
-      <c r="J79" s="146"/>
-      <c r="K79" s="146"/>
-      <c r="L79" s="146"/>
-      <c r="M79" s="146"/>
+      <c r="D79" s="149"/>
+      <c r="E79" s="149"/>
+      <c r="F79" s="149"/>
+      <c r="G79" s="149"/>
+      <c r="H79" s="149"/>
+      <c r="I79" s="149"/>
+      <c r="J79" s="149"/>
+      <c r="K79" s="149"/>
+      <c r="L79" s="149"/>
+      <c r="M79" s="149"/>
     </row>
     <row r="80" spans="1:13" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A80" s="34" t="s">
@@ -22245,21 +22245,21 @@
       <c r="T82" s="28"/>
     </row>
     <row r="83" spans="1:20" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A83" s="146" t="s">
+      <c r="A83" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B83" s="146"/>
-      <c r="C83" s="146" t="s">
+      <c r="B83" s="149"/>
+      <c r="C83" s="149" t="s">
         <v>61</v>
       </c>
-      <c r="D83" s="146"/>
-      <c r="E83" s="146"/>
-      <c r="F83" s="146"/>
-      <c r="G83" s="146"/>
-      <c r="H83" s="146"/>
-      <c r="I83" s="146"/>
-      <c r="J83" s="146"/>
-      <c r="K83" s="146"/>
+      <c r="D83" s="149"/>
+      <c r="E83" s="149"/>
+      <c r="F83" s="149"/>
+      <c r="G83" s="149"/>
+      <c r="H83" s="149"/>
+      <c r="I83" s="149"/>
+      <c r="J83" s="149"/>
+      <c r="K83" s="149"/>
       <c r="M83" s="28"/>
       <c r="N83" s="28"/>
       <c r="O83" s="28"/>
@@ -22317,24 +22317,24 @@
       <c r="L86" s="21"/>
     </row>
     <row r="87" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A87" s="146" t="s">
+      <c r="A87" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B87" s="146"/>
-      <c r="C87" s="147" t="s">
+      <c r="B87" s="149"/>
+      <c r="C87" s="148" t="s">
         <v>61</v>
       </c>
-      <c r="D87" s="147"/>
-      <c r="E87" s="147"/>
-      <c r="F87" s="147"/>
-      <c r="G87" s="147"/>
-      <c r="H87" s="147"/>
-      <c r="I87" s="147"/>
-      <c r="J87" s="147"/>
-      <c r="K87" s="147"/>
-      <c r="L87" s="147"/>
-      <c r="M87" s="147"/>
-      <c r="N87" s="147"/>
+      <c r="D87" s="148"/>
+      <c r="E87" s="148"/>
+      <c r="F87" s="148"/>
+      <c r="G87" s="148"/>
+      <c r="H87" s="148"/>
+      <c r="I87" s="148"/>
+      <c r="J87" s="148"/>
+      <c r="K87" s="148"/>
+      <c r="L87" s="148"/>
+      <c r="M87" s="148"/>
+      <c r="N87" s="148"/>
     </row>
     <row r="88" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A88" s="34" t="s">
@@ -22385,24 +22385,24 @@
       <c r="L90" s="21"/>
     </row>
     <row r="91" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A91" s="146" t="s">
+      <c r="A91" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B91" s="146"/>
-      <c r="C91" s="146" t="s">
+      <c r="B91" s="149"/>
+      <c r="C91" s="149" t="s">
         <v>61</v>
       </c>
-      <c r="D91" s="146"/>
-      <c r="E91" s="146"/>
-      <c r="F91" s="146"/>
-      <c r="G91" s="146"/>
-      <c r="H91" s="146"/>
-      <c r="I91" s="146"/>
-      <c r="J91" s="146"/>
-      <c r="K91" s="146"/>
-      <c r="L91" s="146"/>
-      <c r="M91" s="146"/>
-      <c r="N91" s="146"/>
+      <c r="D91" s="149"/>
+      <c r="E91" s="149"/>
+      <c r="F91" s="149"/>
+      <c r="G91" s="149"/>
+      <c r="H91" s="149"/>
+      <c r="I91" s="149"/>
+      <c r="J91" s="149"/>
+      <c r="K91" s="149"/>
+      <c r="L91" s="149"/>
+      <c r="M91" s="149"/>
+      <c r="N91" s="149"/>
     </row>
     <row r="92" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A92" s="34" t="s">
@@ -22453,24 +22453,24 @@
       <c r="L94" s="21"/>
     </row>
     <row r="95" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A95" s="146" t="s">
+      <c r="A95" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B95" s="146"/>
-      <c r="C95" s="146" t="s">
+      <c r="B95" s="149"/>
+      <c r="C95" s="149" t="s">
         <v>61</v>
       </c>
-      <c r="D95" s="146"/>
-      <c r="E95" s="146"/>
-      <c r="F95" s="146"/>
-      <c r="G95" s="146"/>
-      <c r="H95" s="146"/>
-      <c r="I95" s="146"/>
-      <c r="J95" s="146"/>
-      <c r="K95" s="146"/>
-      <c r="L95" s="146"/>
-      <c r="M95" s="146"/>
-      <c r="N95" s="146"/>
+      <c r="D95" s="149"/>
+      <c r="E95" s="149"/>
+      <c r="F95" s="149"/>
+      <c r="G95" s="149"/>
+      <c r="H95" s="149"/>
+      <c r="I95" s="149"/>
+      <c r="J95" s="149"/>
+      <c r="K95" s="149"/>
+      <c r="L95" s="149"/>
+      <c r="M95" s="149"/>
+      <c r="N95" s="149"/>
     </row>
     <row r="96" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A96" s="34" t="s">
@@ -22496,18 +22496,18 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A57:L57"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="A43:L47"/>
-    <mergeCell ref="A48:L48"/>
-    <mergeCell ref="A49:L49"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A53:L53"/>
-    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A89:L89"/>
+    <mergeCell ref="A91:B91"/>
+    <mergeCell ref="C91:N91"/>
+    <mergeCell ref="A93:L93"/>
+    <mergeCell ref="A95:B95"/>
+    <mergeCell ref="C95:N95"/>
+    <mergeCell ref="A81:L81"/>
+    <mergeCell ref="A83:B83"/>
+    <mergeCell ref="C83:K83"/>
+    <mergeCell ref="A85:L85"/>
+    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="C87:N87"/>
     <mergeCell ref="A79:B79"/>
     <mergeCell ref="C79:M79"/>
     <mergeCell ref="A59:B59"/>
@@ -22521,18 +22521,18 @@
     <mergeCell ref="A75:B75"/>
     <mergeCell ref="C75:K75"/>
     <mergeCell ref="A77:L77"/>
-    <mergeCell ref="A81:L81"/>
-    <mergeCell ref="A83:B83"/>
-    <mergeCell ref="C83:K83"/>
-    <mergeCell ref="A85:L85"/>
-    <mergeCell ref="A87:B87"/>
-    <mergeCell ref="C87:N87"/>
-    <mergeCell ref="A89:L89"/>
-    <mergeCell ref="A91:B91"/>
-    <mergeCell ref="C91:N91"/>
-    <mergeCell ref="A93:L93"/>
-    <mergeCell ref="A95:B95"/>
-    <mergeCell ref="C95:N95"/>
+    <mergeCell ref="A57:L57"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A43:L47"/>
+    <mergeCell ref="A48:L48"/>
+    <mergeCell ref="A49:L49"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A53:L53"/>
+    <mergeCell ref="A55:B55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
@@ -22578,44 +22578,44 @@
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" ht="21" customHeight="1">
-      <c r="A2" s="140" t="s">
+      <c r="A2" s="139" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="140"/>
-      <c r="C2" s="140"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="140"/>
-      <c r="F2" s="140"/>
-      <c r="G2" s="140"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="140"/>
-      <c r="J2" s="140"/>
-      <c r="K2" s="140"/>
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="139"/>
+      <c r="I2" s="139"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="139"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12" s="6" customFormat="1" ht="21.6" customHeight="1">
-      <c r="A3" s="141" t="s">
+      <c r="A3" s="140" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="142" t="s">
+      <c r="B3" s="141" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="142"/>
-      <c r="E3" s="142"/>
-      <c r="F3" s="142" t="s">
+      <c r="C3" s="141"/>
+      <c r="D3" s="141"/>
+      <c r="E3" s="141"/>
+      <c r="F3" s="141" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="142"/>
-      <c r="H3" s="142"/>
-      <c r="I3" s="142"/>
-      <c r="J3" s="142" t="s">
+      <c r="G3" s="141"/>
+      <c r="H3" s="141"/>
+      <c r="I3" s="141"/>
+      <c r="J3" s="141" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="142"/>
+      <c r="K3" s="141"/>
     </row>
     <row r="4" spans="1:12" s="6" customFormat="1" ht="54" customHeight="1">
-      <c r="A4" s="141"/>
+      <c r="A4" s="140"/>
       <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
@@ -23258,99 +23258,99 @@
     </row>
     <row r="40" spans="1:17" ht="21.95" customHeight="1"/>
     <row r="43" spans="1:17" ht="21.75" customHeight="1">
-      <c r="A43" s="148" t="s">
+      <c r="A43" s="146" t="s">
         <v>56</v>
       </c>
-      <c r="B43" s="143"/>
-      <c r="C43" s="143"/>
-      <c r="D43" s="143"/>
-      <c r="E43" s="143"/>
-      <c r="F43" s="143"/>
-      <c r="G43" s="143"/>
-      <c r="H43" s="143"/>
-      <c r="I43" s="143"/>
-      <c r="J43" s="143"/>
-      <c r="K43" s="143"/>
-      <c r="L43" s="143"/>
+      <c r="B43" s="142"/>
+      <c r="C43" s="142"/>
+      <c r="D43" s="142"/>
+      <c r="E43" s="142"/>
+      <c r="F43" s="142"/>
+      <c r="G43" s="142"/>
+      <c r="H43" s="142"/>
+      <c r="I43" s="142"/>
+      <c r="J43" s="142"/>
+      <c r="K43" s="142"/>
+      <c r="L43" s="142"/>
     </row>
     <row r="44" spans="1:17" ht="21.75" customHeight="1">
-      <c r="A44" s="143"/>
-      <c r="B44" s="143"/>
-      <c r="C44" s="143"/>
-      <c r="D44" s="143"/>
-      <c r="E44" s="143"/>
-      <c r="F44" s="143"/>
-      <c r="G44" s="143"/>
-      <c r="H44" s="143"/>
-      <c r="I44" s="143"/>
-      <c r="J44" s="143"/>
-      <c r="K44" s="143"/>
-      <c r="L44" s="143"/>
+      <c r="A44" s="142"/>
+      <c r="B44" s="142"/>
+      <c r="C44" s="142"/>
+      <c r="D44" s="142"/>
+      <c r="E44" s="142"/>
+      <c r="F44" s="142"/>
+      <c r="G44" s="142"/>
+      <c r="H44" s="142"/>
+      <c r="I44" s="142"/>
+      <c r="J44" s="142"/>
+      <c r="K44" s="142"/>
+      <c r="L44" s="142"/>
       <c r="N44" s="33"/>
       <c r="O44" s="33"/>
       <c r="P44" s="33"/>
       <c r="Q44" s="33"/>
     </row>
     <row r="45" spans="1:17" ht="21.75" customHeight="1">
-      <c r="A45" s="143"/>
-      <c r="B45" s="143"/>
-      <c r="C45" s="143"/>
-      <c r="D45" s="143"/>
-      <c r="E45" s="143"/>
-      <c r="F45" s="143"/>
-      <c r="G45" s="143"/>
-      <c r="H45" s="143"/>
-      <c r="I45" s="143"/>
-      <c r="J45" s="143"/>
-      <c r="K45" s="143"/>
-      <c r="L45" s="143"/>
+      <c r="A45" s="142"/>
+      <c r="B45" s="142"/>
+      <c r="C45" s="142"/>
+      <c r="D45" s="142"/>
+      <c r="E45" s="142"/>
+      <c r="F45" s="142"/>
+      <c r="G45" s="142"/>
+      <c r="H45" s="142"/>
+      <c r="I45" s="142"/>
+      <c r="J45" s="142"/>
+      <c r="K45" s="142"/>
+      <c r="L45" s="142"/>
       <c r="P45" s="33"/>
       <c r="Q45" s="33"/>
     </row>
     <row r="46" spans="1:17" ht="21.75" customHeight="1">
-      <c r="A46" s="143"/>
-      <c r="B46" s="143"/>
-      <c r="C46" s="143"/>
-      <c r="D46" s="143"/>
-      <c r="E46" s="143"/>
-      <c r="F46" s="143"/>
-      <c r="G46" s="143"/>
-      <c r="H46" s="143"/>
-      <c r="I46" s="143"/>
-      <c r="J46" s="143"/>
-      <c r="K46" s="143"/>
-      <c r="L46" s="143"/>
+      <c r="A46" s="142"/>
+      <c r="B46" s="142"/>
+      <c r="C46" s="142"/>
+      <c r="D46" s="142"/>
+      <c r="E46" s="142"/>
+      <c r="F46" s="142"/>
+      <c r="G46" s="142"/>
+      <c r="H46" s="142"/>
+      <c r="I46" s="142"/>
+      <c r="J46" s="142"/>
+      <c r="K46" s="142"/>
+      <c r="L46" s="142"/>
       <c r="P46" s="33"/>
     </row>
     <row r="47" spans="1:17" ht="78.75" customHeight="1">
-      <c r="A47" s="143"/>
-      <c r="B47" s="143"/>
-      <c r="C47" s="143"/>
-      <c r="D47" s="143"/>
-      <c r="E47" s="143"/>
-      <c r="F47" s="143"/>
-      <c r="G47" s="143"/>
-      <c r="H47" s="143"/>
-      <c r="I47" s="143"/>
-      <c r="J47" s="143"/>
-      <c r="K47" s="143"/>
-      <c r="L47" s="143"/>
+      <c r="A47" s="142"/>
+      <c r="B47" s="142"/>
+      <c r="C47" s="142"/>
+      <c r="D47" s="142"/>
+      <c r="E47" s="142"/>
+      <c r="F47" s="142"/>
+      <c r="G47" s="142"/>
+      <c r="H47" s="142"/>
+      <c r="I47" s="142"/>
+      <c r="J47" s="142"/>
+      <c r="K47" s="142"/>
+      <c r="L47" s="142"/>
     </row>
     <row r="48" spans="1:17" ht="42" customHeight="1">
-      <c r="A48" s="149" t="s">
+      <c r="A48" s="147" t="s">
         <v>93</v>
       </c>
-      <c r="B48" s="149"/>
-      <c r="C48" s="149"/>
-      <c r="D48" s="149"/>
-      <c r="E48" s="149"/>
-      <c r="F48" s="149"/>
-      <c r="G48" s="149"/>
-      <c r="H48" s="149"/>
-      <c r="I48" s="149"/>
-      <c r="J48" s="149"/>
-      <c r="K48" s="149"/>
-      <c r="L48" s="149"/>
+      <c r="B48" s="147"/>
+      <c r="C48" s="147"/>
+      <c r="D48" s="147"/>
+      <c r="E48" s="147"/>
+      <c r="F48" s="147"/>
+      <c r="G48" s="147"/>
+      <c r="H48" s="147"/>
+      <c r="I48" s="147"/>
+      <c r="J48" s="147"/>
+      <c r="K48" s="147"/>
+      <c r="L48" s="147"/>
     </row>
     <row r="49" spans="1:12" s="21" customFormat="1" ht="30" customHeight="1">
       <c r="A49" s="145" t="s">
@@ -23378,10 +23378,10 @@
       <c r="C50" s="35"/>
     </row>
     <row r="51" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A51" s="147" t="s">
+      <c r="A51" s="148" t="s">
         <v>60</v>
       </c>
-      <c r="B51" s="147"/>
+      <c r="B51" s="148"/>
       <c r="C51" s="34" t="s">
         <v>96</v>
       </c>
@@ -23421,10 +23421,10 @@
       <c r="D54" s="34"/>
     </row>
     <row r="55" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A55" s="147" t="s">
+      <c r="A55" s="148" t="s">
         <v>34</v>
       </c>
-      <c r="B55" s="147"/>
+      <c r="B55" s="148"/>
       <c r="C55" s="34" t="s">
         <v>96</v>
       </c>
@@ -23464,10 +23464,10 @@
       <c r="D58" s="34"/>
     </row>
     <row r="59" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A59" s="146" t="s">
+      <c r="A59" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="146"/>
+      <c r="B59" s="149"/>
       <c r="C59" s="34" t="s">
         <v>66</v>
       </c>
@@ -23507,10 +23507,10 @@
       <c r="D62" s="34"/>
     </row>
     <row r="63" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A63" s="146" t="s">
+      <c r="A63" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B63" s="146"/>
+      <c r="B63" s="149"/>
       <c r="C63" s="34" t="s">
         <v>61</v>
       </c>
@@ -23548,10 +23548,10 @@
       <c r="D66" s="34"/>
     </row>
     <row r="67" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A67" s="146" t="s">
+      <c r="A67" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B67" s="146"/>
+      <c r="B67" s="149"/>
       <c r="C67" s="34" t="s">
         <v>66</v>
       </c>
@@ -23590,10 +23590,10 @@
       <c r="D70" s="34"/>
     </row>
     <row r="71" spans="1:12" s="21" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A71" s="146" t="s">
+      <c r="A71" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B71" s="146"/>
+      <c r="B71" s="149"/>
       <c r="C71" s="34" t="s">
         <v>66</v>
       </c>
@@ -23634,22 +23634,22 @@
       <c r="C74" s="35"/>
     </row>
     <row r="75" spans="1:12" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A75" s="147" t="s">
+      <c r="A75" s="148" t="s">
         <v>34</v>
       </c>
-      <c r="B75" s="147"/>
-      <c r="C75" s="146" t="s">
+      <c r="B75" s="148"/>
+      <c r="C75" s="149" t="s">
         <v>96</v>
       </c>
-      <c r="D75" s="146"/>
-      <c r="E75" s="146"/>
-      <c r="F75" s="146"/>
-      <c r="G75" s="146"/>
-      <c r="H75" s="146"/>
-      <c r="I75" s="146"/>
-      <c r="J75" s="146"/>
-      <c r="K75" s="146"/>
-      <c r="L75" s="146"/>
+      <c r="D75" s="149"/>
+      <c r="E75" s="149"/>
+      <c r="F75" s="149"/>
+      <c r="G75" s="149"/>
+      <c r="H75" s="149"/>
+      <c r="I75" s="149"/>
+      <c r="J75" s="149"/>
+      <c r="K75" s="149"/>
+      <c r="L75" s="149"/>
     </row>
     <row r="76" spans="1:12" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A76" s="34" t="s">
@@ -23685,22 +23685,22 @@
       <c r="D78" s="34"/>
     </row>
     <row r="79" spans="1:12" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A79" s="147" t="s">
+      <c r="A79" s="148" t="s">
         <v>34</v>
       </c>
-      <c r="B79" s="147"/>
-      <c r="C79" s="146" t="s">
+      <c r="B79" s="148"/>
+      <c r="C79" s="149" t="s">
         <v>61</v>
       </c>
-      <c r="D79" s="146"/>
-      <c r="E79" s="146"/>
-      <c r="F79" s="146"/>
-      <c r="G79" s="146"/>
-      <c r="H79" s="146"/>
-      <c r="I79" s="146"/>
-      <c r="J79" s="146"/>
-      <c r="K79" s="146"/>
-      <c r="L79" s="146"/>
+      <c r="D79" s="149"/>
+      <c r="E79" s="149"/>
+      <c r="F79" s="149"/>
+      <c r="G79" s="149"/>
+      <c r="H79" s="149"/>
+      <c r="I79" s="149"/>
+      <c r="J79" s="149"/>
+      <c r="K79" s="149"/>
+      <c r="L79" s="149"/>
     </row>
     <row r="80" spans="1:12" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A80" s="34" t="s">
@@ -23742,22 +23742,22 @@
       <c r="T82" s="28"/>
     </row>
     <row r="83" spans="1:20" s="21" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A83" s="146" t="s">
+      <c r="A83" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B83" s="146"/>
-      <c r="C83" s="146" t="s">
+      <c r="B83" s="149"/>
+      <c r="C83" s="149" t="s">
         <v>96</v>
       </c>
-      <c r="D83" s="146"/>
-      <c r="E83" s="146"/>
-      <c r="F83" s="146"/>
-      <c r="G83" s="146"/>
-      <c r="H83" s="146"/>
-      <c r="I83" s="146"/>
-      <c r="J83" s="146"/>
-      <c r="K83" s="146"/>
-      <c r="L83" s="146"/>
+      <c r="D83" s="149"/>
+      <c r="E83" s="149"/>
+      <c r="F83" s="149"/>
+      <c r="G83" s="149"/>
+      <c r="H83" s="149"/>
+      <c r="I83" s="149"/>
+      <c r="J83" s="149"/>
+      <c r="K83" s="149"/>
+      <c r="L83" s="149"/>
       <c r="M83" s="28"/>
       <c r="N83" s="28"/>
       <c r="O83" s="28"/>
@@ -23817,21 +23817,21 @@
       <c r="L86" s="21"/>
     </row>
     <row r="87" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A87" s="146" t="s">
+      <c r="A87" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B87" s="146"/>
-      <c r="C87" s="146" t="s">
+      <c r="B87" s="149"/>
+      <c r="C87" s="149" t="s">
         <v>61</v>
       </c>
-      <c r="D87" s="146"/>
-      <c r="E87" s="146"/>
-      <c r="F87" s="146"/>
-      <c r="G87" s="146"/>
-      <c r="H87" s="146"/>
-      <c r="I87" s="146"/>
-      <c r="J87" s="146"/>
-      <c r="K87" s="146"/>
+      <c r="D87" s="149"/>
+      <c r="E87" s="149"/>
+      <c r="F87" s="149"/>
+      <c r="G87" s="149"/>
+      <c r="H87" s="149"/>
+      <c r="I87" s="149"/>
+      <c r="J87" s="149"/>
+      <c r="K87" s="149"/>
       <c r="L87" s="21"/>
     </row>
     <row r="88" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
@@ -23883,21 +23883,21 @@
       <c r="L90" s="21"/>
     </row>
     <row r="91" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A91" s="146" t="s">
+      <c r="A91" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B91" s="146"/>
-      <c r="C91" s="146" t="s">
+      <c r="B91" s="149"/>
+      <c r="C91" s="149" t="s">
         <v>61</v>
       </c>
-      <c r="D91" s="146"/>
-      <c r="E91" s="146"/>
-      <c r="F91" s="146"/>
-      <c r="G91" s="146"/>
-      <c r="H91" s="146"/>
-      <c r="I91" s="146"/>
-      <c r="J91" s="146"/>
-      <c r="K91" s="146"/>
+      <c r="D91" s="149"/>
+      <c r="E91" s="149"/>
+      <c r="F91" s="149"/>
+      <c r="G91" s="149"/>
+      <c r="H91" s="149"/>
+      <c r="I91" s="149"/>
+      <c r="J91" s="149"/>
+      <c r="K91" s="149"/>
       <c r="L91" s="21"/>
     </row>
     <row r="92" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
@@ -23949,20 +23949,20 @@
       <c r="L94" s="21"/>
     </row>
     <row r="95" spans="1:20" s="29" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A95" s="146" t="s">
+      <c r="A95" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="B95" s="146"/>
-      <c r="C95" s="146" t="s">
+      <c r="B95" s="149"/>
+      <c r="C95" s="149" t="s">
         <v>61</v>
       </c>
-      <c r="D95" s="146"/>
-      <c r="E95" s="146"/>
-      <c r="F95" s="146"/>
-      <c r="G95" s="146"/>
-      <c r="H95" s="146"/>
-      <c r="I95" s="146"/>
-      <c r="J95" s="146"/>
+      <c r="D95" s="149"/>
+      <c r="E95" s="149"/>
+      <c r="F95" s="149"/>
+      <c r="G95" s="149"/>
+      <c r="H95" s="149"/>
+      <c r="I95" s="149"/>
+      <c r="J95" s="149"/>
       <c r="K95" s="21"/>
       <c r="L95" s="21"/>
     </row>
@@ -23990,18 +23990,18 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A57:L57"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="A43:L47"/>
-    <mergeCell ref="A48:L48"/>
-    <mergeCell ref="A49:L49"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A53:L53"/>
-    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A89:L89"/>
+    <mergeCell ref="A91:B91"/>
+    <mergeCell ref="C91:K91"/>
+    <mergeCell ref="A93:L93"/>
+    <mergeCell ref="A95:B95"/>
+    <mergeCell ref="C95:J95"/>
+    <mergeCell ref="A81:L81"/>
+    <mergeCell ref="A83:B83"/>
+    <mergeCell ref="C83:L83"/>
+    <mergeCell ref="A85:L85"/>
+    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="C87:K87"/>
     <mergeCell ref="A79:B79"/>
     <mergeCell ref="C79:L79"/>
     <mergeCell ref="A59:B59"/>
@@ -24015,18 +24015,18 @@
     <mergeCell ref="A75:B75"/>
     <mergeCell ref="C75:L75"/>
     <mergeCell ref="A77:L77"/>
-    <mergeCell ref="A81:L81"/>
-    <mergeCell ref="A83:B83"/>
-    <mergeCell ref="C83:L83"/>
-    <mergeCell ref="A85:L85"/>
-    <mergeCell ref="A87:B87"/>
-    <mergeCell ref="C87:K87"/>
-    <mergeCell ref="A89:L89"/>
-    <mergeCell ref="A91:B91"/>
-    <mergeCell ref="C91:K91"/>
-    <mergeCell ref="A93:L93"/>
-    <mergeCell ref="A95:B95"/>
-    <mergeCell ref="C95:J95"/>
+    <mergeCell ref="A57:L57"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A43:L47"/>
+    <mergeCell ref="A48:L48"/>
+    <mergeCell ref="A49:L49"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A53:L53"/>
+    <mergeCell ref="A55:B55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="57" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -24133,7 +24133,7 @@
       <c r="Z2" s="46"/>
     </row>
     <row r="3" spans="1:26" ht="15">
-      <c r="A3" s="132">
+      <c r="A3" s="122">
         <v>65</v>
       </c>
       <c r="B3" s="44" t="s">
@@ -24191,7 +24191,7 @@
       <c r="Z3" s="46"/>
     </row>
     <row r="4" spans="1:26" ht="15">
-      <c r="A4" s="133"/>
+      <c r="A4" s="123"/>
       <c r="B4" s="44" t="s">
         <v>134</v>
       </c>
@@ -24235,7 +24235,7 @@
       <c r="Z4" s="46"/>
     </row>
     <row r="5" spans="1:26" ht="15">
-      <c r="A5" s="133"/>
+      <c r="A5" s="123"/>
       <c r="B5" s="44" t="s">
         <v>135</v>
       </c>
@@ -24275,7 +24275,7 @@
       <c r="Z5" s="46"/>
     </row>
     <row r="6" spans="1:26" ht="15">
-      <c r="A6" s="134"/>
+      <c r="A6" s="124"/>
       <c r="B6" s="44" t="s">
         <v>136</v>
       </c>
@@ -25531,7 +25531,7 @@
       <c r="Z30" s="46"/>
     </row>
     <row r="31" spans="1:26" ht="15">
-      <c r="A31" s="135">
+      <c r="A31" s="125">
         <v>66</v>
       </c>
       <c r="B31" s="55" t="s">
@@ -25585,7 +25585,7 @@
       <c r="Z31" s="46"/>
     </row>
     <row r="32" spans="1:26" ht="15">
-      <c r="A32" s="136"/>
+      <c r="A32" s="126"/>
       <c r="B32" s="55" t="s">
         <v>134</v>
       </c>
@@ -25633,7 +25633,7 @@
       <c r="Z32" s="46"/>
     </row>
     <row r="33" spans="1:26" ht="15">
-      <c r="A33" s="136"/>
+      <c r="A33" s="126"/>
       <c r="B33" s="55" t="s">
         <v>135</v>
       </c>
@@ -25679,7 +25679,7 @@
       <c r="Z33" s="46"/>
     </row>
     <row r="34" spans="1:26" ht="15">
-      <c r="A34" s="137"/>
+      <c r="A34" s="127"/>
       <c r="B34" s="55" t="s">
         <v>136</v>
       </c>
@@ -26943,7 +26943,7 @@
       <c r="Z58" s="46"/>
     </row>
     <row r="59" spans="1:26" ht="14.25">
-      <c r="A59" s="128">
+      <c r="A59" s="119">
         <v>67</v>
       </c>
       <c r="B59" s="63" t="s">
@@ -27002,7 +27002,7 @@
       <c r="Z59" s="46"/>
     </row>
     <row r="60" spans="1:26" ht="14.25">
-      <c r="A60" s="129"/>
+      <c r="A60" s="120"/>
       <c r="B60" s="63" t="s">
         <v>134</v>
       </c>
@@ -27034,7 +27034,7 @@
       <c r="Z60" s="46"/>
     </row>
     <row r="61" spans="1:26" ht="14.25">
-      <c r="A61" s="129"/>
+      <c r="A61" s="120"/>
       <c r="B61" s="63" t="s">
         <v>135</v>
       </c>
@@ -27066,7 +27066,7 @@
       <c r="Z61" s="46"/>
     </row>
     <row r="62" spans="1:26" ht="14.25">
-      <c r="A62" s="130"/>
+      <c r="A62" s="121"/>
       <c r="B62" s="63" t="s">
         <v>136</v>
       </c>
@@ -27312,7 +27312,7 @@
       <c r="Z66" s="46"/>
     </row>
     <row r="67" spans="1:26" ht="14.25">
-      <c r="A67" s="128">
+      <c r="A67" s="119">
         <v>67</v>
       </c>
       <c r="B67" s="63" t="s">
@@ -27371,7 +27371,7 @@
       <c r="Z67" s="46"/>
     </row>
     <row r="68" spans="1:26" ht="15">
-      <c r="A68" s="129"/>
+      <c r="A68" s="120"/>
       <c r="B68" s="66" t="s">
         <v>137</v>
       </c>
@@ -27428,7 +27428,7 @@
       <c r="Z68" s="46"/>
     </row>
     <row r="69" spans="1:26" ht="15">
-      <c r="A69" s="130"/>
+      <c r="A69" s="121"/>
       <c r="B69" s="66" t="s">
         <v>138</v>
       </c>
@@ -27578,7 +27578,7 @@
       <c r="Z71" s="46"/>
     </row>
     <row r="72" spans="1:26" ht="14.25">
-      <c r="A72" s="128">
+      <c r="A72" s="119">
         <v>67</v>
       </c>
       <c r="B72" s="63" t="s">
@@ -27637,7 +27637,7 @@
       <c r="Z72" s="46"/>
     </row>
     <row r="73" spans="1:26" ht="15">
-      <c r="A73" s="129"/>
+      <c r="A73" s="120"/>
       <c r="B73" s="63" t="s">
         <v>137</v>
       </c>
@@ -27699,7 +27699,7 @@
       <c r="Z73" s="46"/>
     </row>
     <row r="74" spans="1:26" ht="15">
-      <c r="A74" s="130"/>
+      <c r="A74" s="121"/>
       <c r="B74" s="66" t="s">
         <v>138</v>
       </c>
@@ -27850,7 +27850,7 @@
       <c r="Z76" s="46"/>
     </row>
     <row r="77" spans="1:26" ht="15">
-      <c r="A77" s="128">
+      <c r="A77" s="119">
         <v>67</v>
       </c>
       <c r="B77" s="63" t="s">
@@ -27909,7 +27909,7 @@
       <c r="Z77" s="46"/>
     </row>
     <row r="78" spans="1:26" ht="15">
-      <c r="A78" s="129"/>
+      <c r="A78" s="120"/>
       <c r="B78" s="66" t="s">
         <v>137</v>
       </c>
@@ -27975,7 +27975,7 @@
       <c r="Z78" s="46"/>
     </row>
     <row r="79" spans="1:26" ht="15">
-      <c r="A79" s="130"/>
+      <c r="A79" s="121"/>
       <c r="B79" s="66" t="s">
         <v>138</v>
       </c>
@@ -28127,7 +28127,7 @@
       <c r="Z81" s="46"/>
     </row>
     <row r="82" spans="1:26" ht="15">
-      <c r="A82" s="128">
+      <c r="A82" s="119">
         <v>67</v>
       </c>
       <c r="B82" s="63" t="s">
@@ -28186,7 +28186,7 @@
       <c r="Z82" s="46"/>
     </row>
     <row r="83" spans="1:26" ht="15">
-      <c r="A83" s="129"/>
+      <c r="A83" s="120"/>
       <c r="B83" s="66" t="s">
         <v>137</v>
       </c>
@@ -28252,7 +28252,7 @@
       <c r="Z83" s="46"/>
     </row>
     <row r="84" spans="1:26" ht="15">
-      <c r="A84" s="130"/>
+      <c r="A84" s="121"/>
       <c r="B84" s="66" t="s">
         <v>138</v>
       </c>
@@ -28404,7 +28404,7 @@
       <c r="Z86" s="46"/>
     </row>
     <row r="87" spans="1:26" ht="14.25">
-      <c r="A87" s="128">
+      <c r="A87" s="119">
         <v>67</v>
       </c>
       <c r="B87" s="63" t="s">
@@ -28470,7 +28470,7 @@
       <c r="Z87" s="46"/>
     </row>
     <row r="88" spans="1:26" ht="15">
-      <c r="A88" s="130"/>
+      <c r="A88" s="121"/>
       <c r="B88" s="66" t="s">
         <v>138</v>
       </c>
@@ -28564,7 +28564,7 @@
       <c r="A90" s="72" t="s">
         <v>119</v>
       </c>
-      <c r="B90" s="131" t="s">
+      <c r="B90" s="128" t="s">
         <v>145</v>
       </c>
       <c r="C90" s="73" t="s">
@@ -28622,7 +28622,7 @@
       <c r="A91" s="76">
         <v>68</v>
       </c>
-      <c r="B91" s="124"/>
+      <c r="B91" s="129"/>
       <c r="C91" s="77">
         <v>18</v>
       </c>
@@ -28773,7 +28773,7 @@
       <c r="A94" s="86" t="s">
         <v>119</v>
       </c>
-      <c r="B94" s="123" t="s">
+      <c r="B94" s="130" t="s">
         <v>139</v>
       </c>
       <c r="C94" s="87" t="s">
@@ -28831,7 +28831,7 @@
       <c r="A95" s="76">
         <v>68</v>
       </c>
-      <c r="B95" s="124"/>
+      <c r="B95" s="129"/>
       <c r="C95" s="77">
         <v>35</v>
       </c>
@@ -28982,7 +28982,7 @@
       <c r="A98" s="86" t="s">
         <v>119</v>
       </c>
-      <c r="B98" s="123" t="s">
+      <c r="B98" s="130" t="s">
         <v>140</v>
       </c>
       <c r="C98" s="87" t="s">
@@ -29037,10 +29037,10 @@
       <c r="Z98" s="46"/>
     </row>
     <row r="99" spans="1:26" ht="14.25">
-      <c r="A99" s="125">
+      <c r="A99" s="131">
         <v>68</v>
       </c>
-      <c r="B99" s="124"/>
+      <c r="B99" s="129"/>
       <c r="C99" s="77">
         <v>3</v>
       </c>
@@ -29091,7 +29091,7 @@
       <c r="Z99" s="46"/>
     </row>
     <row r="100" spans="1:26" ht="15">
-      <c r="A100" s="126"/>
+      <c r="A100" s="132"/>
       <c r="B100" s="81" t="s">
         <v>138</v>
       </c>
@@ -29191,7 +29191,7 @@
       <c r="A102" s="86" t="s">
         <v>119</v>
       </c>
-      <c r="B102" s="123" t="s">
+      <c r="B102" s="130" t="s">
         <v>146</v>
       </c>
       <c r="C102" s="87" t="s">
@@ -29246,10 +29246,10 @@
       <c r="Z102" s="46"/>
     </row>
     <row r="103" spans="1:26" ht="15">
-      <c r="A103" s="125">
+      <c r="A103" s="131">
         <v>68</v>
       </c>
-      <c r="B103" s="124"/>
+      <c r="B103" s="129"/>
       <c r="C103" s="77">
         <v>16</v>
       </c>
@@ -29300,7 +29300,7 @@
       <c r="Z103" s="46"/>
     </row>
     <row r="104" spans="1:26" ht="15">
-      <c r="A104" s="126"/>
+      <c r="A104" s="132"/>
       <c r="B104" s="81" t="s">
         <v>138</v>
       </c>
@@ -29583,7 +29583,7 @@
       <c r="A110" s="96" t="s">
         <v>119</v>
       </c>
-      <c r="B110" s="127" t="s">
+      <c r="B110" s="137" t="s">
         <v>145</v>
       </c>
       <c r="C110" s="97" t="s">
@@ -29641,7 +29641,7 @@
       <c r="A111" s="99">
         <v>69</v>
       </c>
-      <c r="B111" s="120"/>
+      <c r="B111" s="134"/>
       <c r="C111" s="100">
         <v>5.25</v>
       </c>
@@ -29782,7 +29782,7 @@
       <c r="A114" s="109" t="s">
         <v>119</v>
       </c>
-      <c r="B114" s="119" t="s">
+      <c r="B114" s="133" t="s">
         <v>139</v>
       </c>
       <c r="C114" s="110" t="s">
@@ -29840,7 +29840,7 @@
       <c r="A115" s="99">
         <v>69</v>
       </c>
-      <c r="B115" s="120"/>
+      <c r="B115" s="134"/>
       <c r="C115" s="100">
         <v>31</v>
       </c>
@@ -29981,7 +29981,7 @@
       <c r="A118" s="109" t="s">
         <v>119</v>
       </c>
-      <c r="B118" s="119" t="s">
+      <c r="B118" s="133" t="s">
         <v>140</v>
       </c>
       <c r="C118" s="110" t="s">
@@ -30036,10 +30036,10 @@
       <c r="Z118" s="46"/>
     </row>
     <row r="119" spans="1:26" ht="14.25">
-      <c r="A119" s="121">
+      <c r="A119" s="135">
         <v>69</v>
       </c>
-      <c r="B119" s="120"/>
+      <c r="B119" s="134"/>
       <c r="C119" s="100">
         <v>3.5</v>
       </c>
@@ -30080,7 +30080,7 @@
       <c r="Z119" s="46"/>
     </row>
     <row r="120" spans="1:26" ht="15">
-      <c r="A120" s="122"/>
+      <c r="A120" s="136"/>
       <c r="B120" s="104" t="s">
         <v>138</v>
       </c>
@@ -30180,7 +30180,7 @@
       <c r="A122" s="109" t="s">
         <v>119</v>
       </c>
-      <c r="B122" s="119" t="s">
+      <c r="B122" s="133" t="s">
         <v>146</v>
       </c>
       <c r="C122" s="110" t="s">
@@ -30235,10 +30235,10 @@
       <c r="Z122" s="46"/>
     </row>
     <row r="123" spans="1:26" ht="15">
-      <c r="A123" s="121">
+      <c r="A123" s="135">
         <v>69</v>
       </c>
-      <c r="B123" s="120"/>
+      <c r="B123" s="134"/>
       <c r="C123" s="100">
         <v>14</v>
       </c>
@@ -30260,7 +30260,9 @@
       <c r="I123" s="101">
         <v>11</v>
       </c>
-      <c r="J123" s="101"/>
+      <c r="J123" s="101">
+        <v>11.26</v>
+      </c>
       <c r="K123" s="101"/>
       <c r="L123" s="101"/>
       <c r="M123" s="101"/>
@@ -30279,7 +30281,7 @@
       <c r="Z123" s="46"/>
     </row>
     <row r="124" spans="1:26" ht="15">
-      <c r="A124" s="122"/>
+      <c r="A124" s="136"/>
       <c r="B124" s="104" t="s">
         <v>138</v>
       </c>
@@ -30313,7 +30315,7 @@
       </c>
       <c r="J124" s="104">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>30.402000000000001</v>
       </c>
       <c r="K124" s="104">
         <f t="shared" si="19"/>
@@ -30496,7 +30498,7 @@
       </c>
       <c r="J128" s="115">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>30.402000000000001</v>
       </c>
       <c r="K128" s="115">
         <f t="shared" si="20"/>
@@ -54584,18 +54586,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A77:A79"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="A67:A69"/>
-    <mergeCell ref="A72:A74"/>
-    <mergeCell ref="A82:A84"/>
-    <mergeCell ref="A87:A88"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="B94:B95"/>
-    <mergeCell ref="B98:B99"/>
-    <mergeCell ref="A99:A100"/>
     <mergeCell ref="B122:B123"/>
     <mergeCell ref="A123:A124"/>
     <mergeCell ref="B102:B103"/>
@@ -54604,6 +54594,18 @@
     <mergeCell ref="B114:B115"/>
     <mergeCell ref="B118:B119"/>
     <mergeCell ref="A119:A120"/>
+    <mergeCell ref="A82:A84"/>
+    <mergeCell ref="A87:A88"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="B98:B99"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="A77:A79"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="A67:A69"/>
+    <mergeCell ref="A72:A74"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -55400,44 +55402,44 @@
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" ht="29.25">
-      <c r="A2" s="140" t="s">
+      <c r="A2" s="139" t="s">
         <v>147</v>
       </c>
-      <c r="B2" s="140"/>
-      <c r="C2" s="140"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="140"/>
-      <c r="F2" s="140"/>
-      <c r="G2" s="140"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="140"/>
-      <c r="J2" s="140"/>
-      <c r="K2" s="140"/>
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="139"/>
+      <c r="I2" s="139"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="139"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12" s="6" customFormat="1" ht="23.25">
-      <c r="A3" s="141" t="s">
+      <c r="A3" s="140" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="142" t="s">
+      <c r="B3" s="141" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="142"/>
-      <c r="E3" s="142"/>
-      <c r="F3" s="142" t="s">
+      <c r="C3" s="141"/>
+      <c r="D3" s="141"/>
+      <c r="E3" s="141"/>
+      <c r="F3" s="141" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="142"/>
-      <c r="H3" s="142"/>
-      <c r="I3" s="142"/>
-      <c r="J3" s="142" t="s">
+      <c r="G3" s="141"/>
+      <c r="H3" s="141"/>
+      <c r="I3" s="141"/>
+      <c r="J3" s="141" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="142"/>
+      <c r="K3" s="141"/>
     </row>
     <row r="4" spans="1:12" s="6" customFormat="1" ht="46.5">
-      <c r="A4" s="141"/>
+      <c r="A4" s="140"/>
       <c r="B4" s="5" t="s">
         <v>6</v>
       </c>

</xml_diff>